<commit_message>
Update UI with new logo and improved design
- Added Ask MOH WingMan logo from uploads folder
- Updated color scheme to blue (#356CA4) and beige (#D4A574)
- Improved typography and spacing for better readability
- Made AI toggle more compact and professional
- Enhanced button styles with flatter, government-standard design
- Simplified upload box with cleaner borders and shadows
- Updated background gradient to diagonal blue-to-beige
- Removed AI-Powered badge from header for cleaner look
- Overall UI/UX improvements for modern government website aesthetic
</commit_message>
<xml_diff>
--- a/sample_questions.xlsx
+++ b/sample_questions.xlsx
@@ -1,88 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
-  <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45E595EB-79FA-499B-BA95-C8B6C06C8B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Question</t>
-  </si>
-  <si>
-    <t>"Dear MOH,
-I would like to enquire whether it is a regulatory requirement for acute hospitals to provide and complete a second financial counselling session within 48 hours upon a patient’s admission, if the patient first enters through the Emergency Department and is subsequently admitted to a ward.
-I came across this information from the following MOH webpage:
-https://www.moh.gov.sg/newsroom/helping-patients-understand-hospital-charges
-However, after reviewing the Healthcare Services Act 2020 (Acute Hospital Service), I was unable to find any reference to the 48-hour requirement. Could you please clarify when the hospital is required to complete the CareCost form for such patients, and whether the 48-hour rule is still applicable in this context?
-Attached is a reference document for your kind attention.
-Thank you, and I look forward to your clarification.
-Best regards
-Kenzo"</t>
-  </si>
-  <si>
-    <t>I recently called 1777 for an ambulance for my grandma who suffered a fall to the nearest hospital. 
-The dispatch went to Carewell Ambulances, and I would like to provide feedback on the entire experience.
-Firstly the cost is absurd for a private ambulance, $260 excluding GST, and for the ambulance to arrive nearly 45 mins later. I called at 8.17pm and they arrived at 9.15pm. if I had called 995 and they deemed it not an emergency I would have paid less. This feels like I am being punished for trying to adhere to the 'non emergency' protocol. 
-Secondly the ambulance arrived with 2 uncles who didn't seem strong enough to carry my grandma (which I explicitly stated was at least 80 kgs during the call) on to the gurney, and in the process of doing that caused her to wail in pain. I also asked whether paramedics will be assigned in the ambulance during the call, both drivers did not look like one. The operator also told me that the ambulance is nearby my pick up location when asking whether I accept the price,which was given as a range.
-Ultimately she arrived at the hospital, which was less than 10 mins drive from pick up location, but I just felt the entire process feels punishing, and doesn't make sense to me. I hope MOH reviews it's PAOs and 1777 policy, as it stands the entire process is laughable and feels neglected.</t>
-  </si>
-  <si>
-    <t>My name is Henrique Peres Caixeta Silva and I was recently admitted at Sayang Wellness Center - Institute of Mental Health (Block 2, Level 4), where I spent one week. 
-Here’s a few things I personally think you could improve based on my own experience:
-Have more food/snacks available for the patients. I actually starved the first days (without external food) since I could not adapt to the Asian neither the western options offered.
-Have more motivated employees. Besides Danny, Cecilia and Jolie, I have no memory of others being very nice to me, on the contrary, some were rude especially during night shift when I was in a most vulnerable position. The English barrier was a problem since it’s not my first language (português is my first language), and sometimes communication wasn’t clear.
-Have someone to adjust the patient air conditioning. The controls/buttons are unnecessary complicated.
-It was freezing the first day and super warm by the end of the week. 
-Have eye mask and ear plugs (like those given by airlines during long haul flights) available for the patients. The amount of noise (doors slamming, and other sounds) and the non-existing black out curtains makes sleeping extra difficult.
-Serve peeled fruits. It’s not reasonable to serve an inteire orange since knives are not allowed, for example.
-My blood pressure was high during my whole stay (specially because of sleep deprivation and stress), and I don’t recall having any medications for high blood pressure. 
-Also, unfortunately, there’s no direct sunlight into the rooms I stayed in, what made my biological clock unbalanced. Fortunately, my family was able to fly from Brazil and provide the necessary support. I was then authorized to go outside with my mom/sister, and this was fundamental for my recovery. 
-On a positive note, I must mention the extraordinary Dr. Peter Chiu and the Osler Health International, where I first sought help for my insomnia/jet lagged problems. I wish I had a physician in Brazil like Dr. Peter Chiu.</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -93,7 +52,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -101,47 +60,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -220,6 +150,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -254,6 +185,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -288,20 +220,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -423,40 +351,128 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="98.42578125" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A6"/>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="321">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="275.25">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="409.6">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Question</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str" xml:space="preserve">
+        <v xml:space="preserve">"Dear MOH,_x000d_
+_x000d_
+I would like to enquire whether it is a regulatory requirement for acute hospitals to provide and complete a second financial counselling session within 48 hours upon a patient’s admission, if the patient first enters through the Emergency Department and is subsequently admitted to a ward._x000d_
+_x000d_
+I came across this information from the following MOH webpage:_x000d_
+https://www.moh.gov.sg/newsroom/helping-patients-understand-hospital-charges_x000d_
+_x000d_
+However, after reviewing the Healthcare Services Act 2020 (Acute Hospital Service), I was unable to find any reference to the 48-hour requirement. Could you please clarify when the hospital is required to complete the CareCost form for such patients, and whether the 48-hour rule is still applicable in this context?_x000d_
+_x000d_
+Attached is a reference document for your kind attention._x000d_
+_x000d_
+Thank you, and I look forward to your clarification._x000d_
+_x000d_
+Best regards_x000d_
+Kenzo"</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str" xml:space="preserve">
+        <v xml:space="preserve">I recently called 1777 for an ambulance for my grandma who suffered a fall to the nearest hospital. _x000d_
+_x000d_
+The dispatch went to Carewell Ambulances, and I would like to provide feedback on the entire experience._x000d_
+_x000d_
+Firstly the cost is absurd for a private ambulance, $260 excluding GST, and for the ambulance to arrive nearly 45 mins later. I called at 8.17pm and they arrived at 9.15pm. if I had called 995 and they deemed it not an emergency I would have paid less. This feels like I am being punished for trying to adhere to the 'non emergency' protocol. _x000d_
+_x000d_
+Secondly the ambulance arrived with 2 uncles who didn't seem strong enough to carry my grandma (which I explicitly stated was at least 80 kgs during the call) on to the gurney, and in the process of doing that caused her to wail in pain. I also asked whether paramedics will be assigned in the ambulance during the call, both drivers did not look like one. The operator also told me that the ambulance is nearby my pick up location when asking whether I accept the price,which was given as a range._x000d_
+_x000d_
+Ultimately she arrived at the hospital, which was less than 10 mins drive from pick up location, but I just felt the entire process feels punishing, and doesn't make sense to me. I hope MOH reviews it's PAOs and 1777 policy, as it stands the entire process is laughable and feels neglected.</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str" xml:space="preserve">
+        <v xml:space="preserve">My name is Henrique Peres Caixeta Silva and I was recently admitted at Sayang Wellness Center - Institute of Mental Health (Block 2, Level 4), where I spent one week. _x000d_
+_x000d_
+Here’s a few things I personally think you could improve based on my own experience:_x000d_
+_x000d_
+Have more food/snacks available for the patients. I actually starved the first days (without external food) since I could not adapt to the Asian neither the western options offered._x000d_
+_x000d_
+Have more motivated employees. Besides Danny, Cecilia and Jolie, I have no memory of others being very nice to me, on the contrary, some were rude especially during night shift when I was in a most vulnerable position. The English barrier was a problem since it’s not my first language (português is my first language), and sometimes communication wasn’t clear._x000d_
+_x000d_
+Have someone to adjust the patient air conditioning. The controls/buttons are unnecessary complicated._x000d_
+It was freezing the first day and super warm by the end of the week. _x000d_
+_x000d_
+Have eye mask and ear plugs (like those given by airlines during long haul flights) available for the patients. The amount of noise (doors slamming, and other sounds) and the non-existing black out curtains makes sleeping extra difficult._x000d_
+_x000d_
+Serve peeled fruits. It’s not reasonable to serve an inteire orange since knives are not allowed, for example._x000d_
+_x000d_
+My blood pressure was high during my whole stay (specially because of sleep deprivation and stress), and I don’t recall having any medications for high blood pressure. _x000d_
+_x000d_
+Also, unfortunately, there’s no direct sunlight into the rooms I stayed in, what made my biological clock unbalanced. Fortunately, my family was able to fly from Brazil and provide the necessary support. I was then authorized to go outside with my mom/sister, and this was fundamental for my recovery. _x000d_
+_x000d_
+On a positive note, I must mention the extraordinary Dr. Peter Chiu and the Osler Health International, where I first sought help for my insomnia/jet lagged problems. I wish I had a physician in Brazil like Dr. Peter Chiu.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>You guys dunno what you all are doing. please improve and ask your manager call me.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Stupid, idiot. I am angry</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>